<commit_message>
Corrige etiqueta resta y agrega seccion Documentos Fuente (practica fija)
</commit_message>
<xml_diff>
--- a/finanzas/informes_semanales/Informe_Financiero_Semanal_Global_Solutions_07Ago2026.xlsx
+++ b/finanzas/informes_semanales/Informe_Financiero_Semanal_Global_Solutions_07Ago2026.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="90">
   <si>
     <t xml:space="preserve">INFORME FINANCIERO SEMANAL — GLOBAL SOLUTIONS SPA — AL 7 AGO 2026</t>
   </si>
@@ -118,7 +118,7 @@
     <t xml:space="preserve">Facturas emitidas pendientes de pago</t>
   </si>
   <si>
-    <t xml:space="preserve">Facturas por emitir (ventas reales − ya facturado)</t>
+    <t xml:space="preserve">Facturas por emitir (ventas reales menos lo facturado)</t>
   </si>
   <si>
     <t xml:space="preserve">— por cliente —</t>
@@ -173,6 +173,123 @@
   </si>
   <si>
     <t xml:space="preserve">Saldo Copec: no aplica — es reembolso directo a Pablo Riquelme vía tarjeta personal, no tiene saldo prepago propio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOCUMENTOS FUENTE DE ESTE INFORME (entregar siempre esta lista)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha/Período</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usado para</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CartolaProvisoria-000037767310-0004-20260807.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartola bancaria Santander</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31/07 al 07/08/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo Santander, egresos categorizados, ingresos factoring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imagen portal Esmax/Aramco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo tarjeta prepago</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07-08-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo Aramco real ($4.977+$91.430)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imagen app Copec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compras Copec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04 y 05-08-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contexto combustible Copec (sin saldo prepago, es reembolso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transacciones__10_.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detalle transacciones Aramco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agosto 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consumo real por patente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">export__68_.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eventos GPS (trip/stop/geofence)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01,03-07/08/2026 (+15,30,31/07)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar servicios "asignado" contra actividad real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RCV_VENTA_78303134-5_202608.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RCV Venta SII</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facturas emitidas del mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RCV_COMPRA_REGISTRO_78303134-5_202608.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RCV Compra SII</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cruce de proveedores/categorización</t>
+  </si>
+  <si>
+    <t xml:space="preserve">servicios_piloto (Supabase)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base de datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventas reales por servicio y cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kaptura_caja (Supabase)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Egresos categorizados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kaptura_cuentas_por_cobrar (Supabase)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Julio 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CxC pendientes de julio</t>
   </si>
 </sst>
 </file>
@@ -350,7 +467,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -405,6 +522,10 @@
     </xf>
     <xf numFmtId="165" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -659,7 +780,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D66"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -1080,8 +1201,170 @@
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
     </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B55" s="3"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D57" s="14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D58" s="14" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D59" s="14" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D60" s="14" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D61" s="14" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B62" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D62" s="14" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B63" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C63" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D63" s="14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D64" s="14" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C65" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D65" s="14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C66" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D66" s="14" t="s">
+        <v>89</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A4:D4"/>
@@ -1098,6 +1381,7 @@
     <mergeCell ref="A52:D52"/>
     <mergeCell ref="A53:D53"/>
     <mergeCell ref="A54:D54"/>
+    <mergeCell ref="A55:D55"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Agrega pago INCOFIN a facturas Serlogin (26+29) al Informe Semanal
</commit_message>
<xml_diff>
--- a/finanzas/informes_semanales/Informe_Financiero_Semanal_Global_Solutions_07Ago2026.xlsx
+++ b/finanzas/informes_semanales/Informe_Financiero_Semanal_Global_Solutions_07Ago2026.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="85">
   <si>
     <t xml:space="preserve">INFORME FINANCIERO SEMANAL</t>
   </si>
@@ -110,7 +110,16 @@
     <t xml:space="preserve">Facturas emitidas (folio 30, Sollem, bruto)</t>
   </si>
   <si>
-    <t xml:space="preserve">Facturas pagadas en cuenta (neto, factoring INCOFIN 04-08)</t>
+    <t xml:space="preserve">Facturas emitidas (folios 26+29, Serlogin, bruto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facturas pagadas en cuenta — Sollem (neto, factoring INCOFIN 04-08)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facturas pagadas en cuenta — Serlogin (neto, factoring INCOFIN 04-08)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total pagado por factoring esta semana (Sollem + Serlogin)</t>
   </si>
   <si>
     <t xml:space="preserve">Facturas emitidas pendientes de pago</t>
@@ -230,16 +239,28 @@
     <t xml:space="preserve">RCV Venta agosto. CONFIRMADO con factura PDF: es cierre de JULIO (GDs 24342,24343), no venta de agosto — no se resta de Ventas Agosto</t>
   </si>
   <si>
+    <t xml:space="preserve">Facturas emitidas — folios 26+29 Serlogin (bruto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RCV Venta julio, folios 26 ($2.361.912) y 29 ($737.800). Facturado en julio, cobrado en agosto</t>
+  </si>
+  <si>
     <t xml:space="preserve">Facturas pagadas en cuenta (neto, factoring)</t>
   </si>
   <si>
-    <t xml:space="preserve">INCOFIN S.A., cartola 04-08-2026</t>
+    <t xml:space="preserve">INCOFIN S.A., cartola 04-08-2026 — folio 30 Sollem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facturas pagadas en cuenta — Serlogin (neto, factoring)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INCOFIN S.A., cartola 04-08-2026 — folios 26+29 Serlogin, comisión 1,5% ($46.496)</t>
   </si>
   <si>
     <t xml:space="preserve">Facturas emitidas pendientes de pago (agosto)</t>
   </si>
   <si>
-    <t xml:space="preserve">Folio 30 quedó 100% liquidado vía factoring — el descuento de factoring es costo financiero, no saldo impago</t>
+    <t xml:space="preserve">Folio 30 y folios 26+29 quedaron 100% liquidados vía factoring — el descuento de factoring es costo financiero, no saldo impago</t>
   </si>
   <si>
     <t xml:space="preserve">FACTURAS EMITIDAS JULIO, SIN PAGO EN CARTOLA (julio ni agosto)</t>
@@ -772,7 +793,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="55"/>
@@ -1044,7 +1065,7 @@
       </c>
       <c r="B32" s="6" t="n">
         <f aca="false">'Memoria de Cálculo'!$B$30</f>
-        <v>605464</v>
+        <v>3099712</v>
       </c>
       <c r="C32" s="6"/>
     </row>
@@ -1054,128 +1075,158 @@
       </c>
       <c r="B33" s="6" t="n">
         <f aca="false">'Memoria de Cálculo'!$B$31</f>
-        <v>0</v>
+        <v>605464</v>
       </c>
       <c r="C33" s="6"/>
     </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B34" s="10" t="n">
-        <f aca="false">B17</f>
-        <v>9397512.11</v>
-      </c>
-      <c r="C34" s="10"/>
+      <c r="B34" s="6" t="n">
+        <f aca="false">'Memoria de Cálculo'!$B$32</f>
+        <v>3053216</v>
+      </c>
+      <c r="C34" s="6"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B35" s="6" t="n">
-        <f aca="false">('Memoria de Cálculo'!$B$11+'Memoria de Cálculo'!$B$12)*(1+'Memoria de Cálculo'!$B$4)</f>
-        <v>6568083.62</v>
-      </c>
-      <c r="C35" s="6"/>
+      <c r="B35" s="8" t="n">
+        <f aca="false">'Memoria de Cálculo'!$B$31+'Memoria de Cálculo'!$B$32</f>
+        <v>3658680</v>
+      </c>
+      <c r="C35" s="8"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
         <v>33</v>
       </c>
       <c r="B36" s="6" t="n">
-        <f aca="false">('Memoria de Cálculo'!$B$13+'Memoria de Cálculo'!$B$14)*(1+'Memoria de Cálculo'!$B$4)</f>
-        <v>1258628.49</v>
+        <f aca="false">'Memoria de Cálculo'!$B$33</f>
+        <v>0</v>
       </c>
       <c r="C36" s="6"/>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="B37" s="6" t="n">
-        <f aca="false">('Memoria de Cálculo'!$B$15+'Memoria de Cálculo'!$B$16)*(1+'Memoria de Cálculo'!$B$4)</f>
-        <v>1071000</v>
-      </c>
-      <c r="C37" s="6"/>
+      <c r="B37" s="10" t="n">
+        <f aca="false">B17</f>
+        <v>9397512.11</v>
+      </c>
+      <c r="C37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
         <v>35</v>
       </c>
       <c r="B38" s="6" t="n">
+        <f aca="false">('Memoria de Cálculo'!$B$11+'Memoria de Cálculo'!$B$12)*(1+'Memoria de Cálculo'!$B$4)</f>
+        <v>6568083.62</v>
+      </c>
+      <c r="C38" s="6"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B39" s="6" t="n">
+        <f aca="false">('Memoria de Cálculo'!$B$13+'Memoria de Cálculo'!$B$14)*(1+'Memoria de Cálculo'!$B$4)</f>
+        <v>1258628.49</v>
+      </c>
+      <c r="C39" s="6"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B40" s="6" t="n">
+        <f aca="false">('Memoria de Cálculo'!$B$15+'Memoria de Cálculo'!$B$16)*(1+'Memoria de Cálculo'!$B$4)</f>
+        <v>1071000</v>
+      </c>
+      <c r="C40" s="6"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B41" s="6" t="n">
         <f aca="false">('Memoria de Cálculo'!$B$17+'Memoria de Cálculo'!$B$18)*(1+'Memoria de Cálculo'!$B$4)</f>
         <v>499800</v>
       </c>
-      <c r="C38" s="6"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="C41" s="6"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B42" s="5" t="s">
+      <c r="B44" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C42" s="14" t="n">
-        <f aca="false">'Memoria de Cálculo'!$B$34</f>
+      <c r="C44" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C45" s="14" t="n">
+        <f aca="false">'Memoria de Cálculo'!$B$36</f>
         <v>690200</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C43" s="14" t="n">
-        <f aca="false">'Memoria de Cálculo'!$B$35</f>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C46" s="14" t="n">
+        <f aca="false">'Memoria de Cálculo'!$B$37</f>
         <v>1428000</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B44" s="15"/>
-      <c r="C44" s="10" t="n">
-        <f aca="false">C42+C43</f>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47" s="15"/>
+      <c r="C47" s="10" t="n">
+        <f aca="false">C45+C46</f>
         <v>2118200</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-    </row>
-    <row r="47" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="B47" s="16"/>
-      <c r="C47" s="16"/>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+    </row>
+    <row r="50" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B50" s="16"/>
+      <c r="C50" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="29">
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
@@ -1199,9 +1250,12 @@
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="A50:C50"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1218,7 +1272,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
@@ -1228,21 +1282,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B4" s="18" t="n">
         <v>0.19</v>
@@ -1250,7 +1304,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1263,118 +1317,118 @@
         <v>303760</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B8" s="19" t="n">
         <v>96407</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B11" s="19" t="n">
         <v>3847555</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B12" s="19" t="n">
         <v>1671843</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B13" s="19" t="n">
         <v>481634</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B14" s="19" t="n">
         <v>576037</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B15" s="19" t="n">
         <v>450000</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B16" s="19" t="n">
         <v>450000</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B17" s="19" t="n">
         <v>420000</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B18" s="18" t="n">
         <v>0</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -1387,7 +1441,7 @@
         <v>2600000</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1398,7 +1452,7 @@
         <v>4193196</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1409,7 +1463,7 @@
         <v>87453</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1420,7 +1474,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1431,7 +1485,7 @@
         <v>1257072</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1442,76 +1496,98 @@
         <v>50000</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B29" s="19" t="n">
         <v>624512</v>
       </c>
       <c r="C29" s="20" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B30" s="19" t="n">
-        <v>605464</v>
+        <v>3099712</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B31" s="18" t="n">
+        <v>74</v>
+      </c>
+      <c r="B31" s="19" t="n">
+        <v>605464</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B32" s="19" t="n">
+        <v>3053216</v>
+      </c>
+      <c r="C32" s="20" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B33" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C31" s="20" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B34" s="19" t="n">
+      <c r="C33" s="20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B36" s="19" t="n">
         <v>690200</v>
       </c>
-      <c r="C34" s="20" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B35" s="19" t="n">
+      <c r="C36" s="20" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B37" s="19" t="n">
         <v>1428000</v>
       </c>
-      <c r="C35" s="20" t="s">
-        <v>77</v>
+      <c r="C37" s="20" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1522,7 +1598,7 @@
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A35:C35"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Separa Copec, corrige label combustible, agrega alerta critica de posible duplicacion de servicios (S-111/S-112 y 8x Lampa sin guia)
</commit_message>
<xml_diff>
--- a/finanzas/informes_semanales/Informe_Financiero_Semanal_Global_Solutions_07Ago2026.xlsx
+++ b/finanzas/informes_semanales/Informe_Financiero_Semanal_Global_Solutions_07Ago2026.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="91">
   <si>
     <t xml:space="preserve">INFORME FINANCIERO SEMANAL</t>
   </si>
@@ -83,7 +83,7 @@
     <t xml:space="preserve">Categoría</t>
   </si>
   <si>
-    <t xml:space="preserve">Combustible (Aramco+Copec vía cartola)</t>
+    <t xml:space="preserve">Combustible — Aramco (top-up vía cartola Santander)</t>
   </si>
   <si>
     <t xml:space="preserve">Remuneraciones</t>
@@ -104,6 +104,12 @@
     <t xml:space="preserve">TOTAL EGRESOS</t>
   </si>
   <si>
+    <t xml:space="preserve">Memo — Combustible Copec (consumo real app, NO incluido en el total de arriba)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota: no se sumó al Total Egresos porque no se confirmó que Pablo Riquelme ya haya sido reembolsado esta semana en la cartola Santander — evita doble conteo sin evidencia.</t>
+  </si>
+  <si>
     <t xml:space="preserve">4. FACTURAS — AGOSTO 2026</t>
   </si>
   <si>
@@ -164,6 +170,12 @@
     <t xml:space="preserve">TOTAL SIN PAGAR</t>
   </si>
   <si>
+    <t xml:space="preserve">⚠ ALERTA — POSIBLE DUPLICACIÓN DE SERVICIOS (sin confirmar, revisar con OPE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Al cruzar contra GPS real (export de eventos trip/stop), se encontró que varios pares de servicios comparten el MISMO camión, MISMO día, MISMA ruta continua sin regreso a base entre uno y otro — ej. S-111/S-112 (Trans Luciano, Codegua, $210.000 c/u, ambos sin num_guia) y 8 servicios distintos con destino "Lampa" a exactamente $306.415 cada uno, también sin num_guia que los distinga. No se puede confirmar si son viajes reales separados o el mismo dato cargado más de una vez. El Total de Ventas de Agosto ($9.397.512) queda marcado como NO CONFIRMADO hasta que se revise.</t>
+  </si>
+  <si>
     <t xml:space="preserve">NOTA IMPORTANTE</t>
   </si>
   <si>
@@ -228,6 +240,12 @@
   </si>
   <si>
     <t xml:space="preserve">kaptura_caja, categorización real cruzada RCV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combustible — Copec (reembolso Pablo Riquelme, separado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App Copec: 04-08 $200.000 + 05-08 $50.000. NO estaba antes visible como línea propia, mezclado en Remuneraciones</t>
   </si>
   <si>
     <t xml:space="preserve">FACTURAS — AGOSTO 2026</t>
@@ -287,7 +305,7 @@
     <numFmt numFmtId="165" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -362,6 +380,23 @@
       <charset val="1"/>
     </font>
     <font>
+      <i val="true"/>
+      <sz val="8"/>
+      <color rgb="FF808080"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FF9C0006"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
@@ -369,7 +404,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -398,6 +433,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -456,7 +497,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -509,11 +550,23 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -521,6 +574,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -529,11 +586,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -560,7 +617,7 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF9C0006"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
@@ -587,7 +644,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFC6EFCE"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFEB9C"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -793,7 +850,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="55"/>
@@ -1034,48 +1091,44 @@
       </c>
       <c r="C27" s="10"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+    <row r="28" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="B28" s="14" t="n">
+        <f aca="false">'Memoria de Cálculo'!$B$27</f>
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B32" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B31" s="6" t="n">
-        <f aca="false">'Memoria de Cálculo'!$B$29</f>
-        <v>624512</v>
-      </c>
-      <c r="C31" s="6"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B32" s="6" t="n">
-        <f aca="false">'Memoria de Cálculo'!$B$30</f>
-        <v>3099712</v>
-      </c>
-      <c r="C32" s="6"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="6" t="n">
-        <f aca="false">'Memoria de Cálculo'!$B$31</f>
-        <v>605464</v>
+        <f aca="false">'Memoria de Cálculo'!$B$30</f>
+        <v>624512</v>
       </c>
       <c r="C33" s="6"/>
     </row>
@@ -1084,20 +1137,20 @@
         <v>31</v>
       </c>
       <c r="B34" s="6" t="n">
+        <f aca="false">'Memoria de Cálculo'!$B$31</f>
+        <v>3099712</v>
+      </c>
+      <c r="C34" s="6"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" s="6" t="n">
         <f aca="false">'Memoria de Cálculo'!$B$32</f>
-        <v>3053216</v>
-      </c>
-      <c r="C34" s="6"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B35" s="8" t="n">
-        <f aca="false">'Memoria de Cálculo'!$B$31+'Memoria de Cálculo'!$B$32</f>
-        <v>3658680</v>
-      </c>
-      <c r="C35" s="8"/>
+        <v>605464</v>
+      </c>
+      <c r="C35" s="6"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
@@ -1105,47 +1158,47 @@
       </c>
       <c r="B36" s="6" t="n">
         <f aca="false">'Memoria de Cálculo'!$B$33</f>
-        <v>0</v>
+        <v>3053216</v>
       </c>
       <c r="C36" s="6"/>
     </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="13" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B37" s="10" t="n">
-        <f aca="false">B17</f>
-        <v>9397512.11</v>
-      </c>
-      <c r="C37" s="10"/>
+      <c r="B37" s="8" t="n">
+        <f aca="false">'Memoria de Cálculo'!$B$32+'Memoria de Cálculo'!$B$33</f>
+        <v>3658680</v>
+      </c>
+      <c r="C37" s="8"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
         <v>35</v>
       </c>
       <c r="B38" s="6" t="n">
-        <f aca="false">('Memoria de Cálculo'!$B$11+'Memoria de Cálculo'!$B$12)*(1+'Memoria de Cálculo'!$B$4)</f>
-        <v>6568083.62</v>
+        <f aca="false">'Memoria de Cálculo'!$B$34</f>
+        <v>0</v>
       </c>
       <c r="C38" s="6"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="s">
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B39" s="6" t="n">
-        <f aca="false">('Memoria de Cálculo'!$B$13+'Memoria de Cálculo'!$B$14)*(1+'Memoria de Cálculo'!$B$4)</f>
-        <v>1258628.49</v>
-      </c>
-      <c r="C39" s="6"/>
+      <c r="B39" s="10" t="n">
+        <f aca="false">B17</f>
+        <v>9397512.11</v>
+      </c>
+      <c r="C39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
         <v>37</v>
       </c>
       <c r="B40" s="6" t="n">
-        <f aca="false">('Memoria de Cálculo'!$B$15+'Memoria de Cálculo'!$B$16)*(1+'Memoria de Cálculo'!$B$4)</f>
-        <v>1071000</v>
+        <f aca="false">('Memoria de Cálculo'!$B$11+'Memoria de Cálculo'!$B$12)*(1+'Memoria de Cálculo'!$B$4)</f>
+        <v>6568083.62</v>
       </c>
       <c r="C40" s="6"/>
     </row>
@@ -1154,79 +1207,113 @@
         <v>38</v>
       </c>
       <c r="B41" s="6" t="n">
+        <f aca="false">('Memoria de Cálculo'!$B$13+'Memoria de Cálculo'!$B$14)*(1+'Memoria de Cálculo'!$B$4)</f>
+        <v>1258628.49</v>
+      </c>
+      <c r="C41" s="6"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B42" s="6" t="n">
+        <f aca="false">('Memoria de Cálculo'!$B$15+'Memoria de Cálculo'!$B$16)*(1+'Memoria de Cálculo'!$B$4)</f>
+        <v>1071000</v>
+      </c>
+      <c r="C42" s="6"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B43" s="6" t="n">
         <f aca="false">('Memoria de Cálculo'!$B$17+'Memoria de Cálculo'!$B$18)*(1+'Memoria de Cálculo'!$B$4)</f>
         <v>499800</v>
       </c>
-      <c r="C41" s="6"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="4" t="s">
+      <c r="C43" s="6"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B44" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5" t="s">
+      <c r="B46" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="C46" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C45" s="14" t="n">
-        <f aca="false">'Memoria de Cálculo'!$B$36</f>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C47" s="17" t="n">
+        <f aca="false">'Memoria de Cálculo'!$B$37</f>
         <v>690200</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C46" s="14" t="n">
-        <f aca="false">'Memoria de Cálculo'!$B$37</f>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C48" s="17" t="n">
+        <f aca="false">'Memoria de Cálculo'!$B$38</f>
         <v>1428000</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="B47" s="15"/>
-      <c r="C47" s="10" t="n">
-        <f aca="false">C45+C46</f>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" s="18"/>
+      <c r="C49" s="10" t="n">
+        <f aca="false">C47+C48</f>
         <v>2118200</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B49" s="3"/>
-      <c r="C49" s="3"/>
-    </row>
-    <row r="50" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="B50" s="16"/>
-      <c r="C50" s="16"/>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+    </row>
+    <row r="52" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="B52" s="19"/>
+      <c r="C52" s="19"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B54" s="3"/>
+      <c r="C54" s="3"/>
+    </row>
+    <row r="55" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B55" s="20"/>
+      <c r="C55" s="20"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="32">
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
@@ -1242,8 +1329,7 @@
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="A29:C29"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
@@ -1253,9 +1339,13 @@
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B41:C41"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="A54:C54"/>
+    <mergeCell ref="A55:C55"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1272,7 +1362,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
@@ -1281,30 +1371,30 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
+      <c r="A1" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B4" s="18" t="n">
+        <v>55</v>
+      </c>
+      <c r="B4" s="22" t="n">
         <v>0.19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1313,122 +1403,122 @@
       <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="23" t="n">
         <v>303760</v>
       </c>
-      <c r="C7" s="20" t="s">
-        <v>53</v>
+      <c r="C7" s="24" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B8" s="19" t="n">
+        <v>58</v>
+      </c>
+      <c r="B8" s="23" t="n">
         <v>96407</v>
       </c>
-      <c r="C8" s="20" t="s">
-        <v>55</v>
+      <c r="C8" s="24" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B11" s="19" t="n">
+        <v>61</v>
+      </c>
+      <c r="B11" s="23" t="n">
         <v>3847555</v>
       </c>
-      <c r="C11" s="20" t="s">
-        <v>58</v>
+      <c r="C11" s="24" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B12" s="19" t="n">
+        <v>63</v>
+      </c>
+      <c r="B12" s="23" t="n">
         <v>1671843</v>
       </c>
-      <c r="C12" s="20" t="s">
-        <v>60</v>
+      <c r="C12" s="24" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B13" s="19" t="n">
+        <v>65</v>
+      </c>
+      <c r="B13" s="23" t="n">
         <v>481634</v>
       </c>
-      <c r="C13" s="20" t="s">
-        <v>58</v>
+      <c r="C13" s="24" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B14" s="19" t="n">
+        <v>66</v>
+      </c>
+      <c r="B14" s="23" t="n">
         <v>576037</v>
       </c>
-      <c r="C14" s="20" t="s">
-        <v>60</v>
+      <c r="C14" s="24" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B15" s="19" t="n">
+        <v>67</v>
+      </c>
+      <c r="B15" s="23" t="n">
         <v>450000</v>
       </c>
-      <c r="C15" s="20" t="s">
-        <v>58</v>
+      <c r="C15" s="24" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B16" s="23" t="n">
+        <v>450000</v>
+      </c>
+      <c r="C16" s="24" t="s">
         <v>64</v>
-      </c>
-      <c r="B16" s="19" t="n">
-        <v>450000</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="B17" s="19" t="n">
+        <v>69</v>
+      </c>
+      <c r="B17" s="23" t="n">
         <v>420000</v>
       </c>
-      <c r="C17" s="20" t="s">
-        <v>58</v>
+      <c r="C17" s="24" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B18" s="18" t="n">
+        <v>70</v>
+      </c>
+      <c r="B18" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="C18" s="20" t="s">
-        <v>60</v>
+      <c r="C18" s="24" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -1437,157 +1527,168 @@
       <c r="A21" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="19" t="n">
+      <c r="B21" s="23" t="n">
         <v>2600000</v>
       </c>
-      <c r="C21" s="20" t="s">
-        <v>68</v>
+      <c r="C21" s="24" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="19" t="n">
+      <c r="B22" s="23" t="n">
         <v>4193196</v>
       </c>
-      <c r="C22" s="20" t="s">
-        <v>68</v>
+      <c r="C22" s="24" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="19" t="n">
+      <c r="B23" s="23" t="n">
         <v>87453</v>
       </c>
-      <c r="C23" s="20" t="s">
-        <v>68</v>
+      <c r="C23" s="24" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="18" t="n">
+      <c r="B24" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="C24" s="20" t="s">
-        <v>68</v>
+      <c r="C24" s="24" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="19" t="n">
+      <c r="B25" s="23" t="n">
         <v>1257072</v>
       </c>
-      <c r="C25" s="20" t="s">
-        <v>68</v>
+      <c r="C25" s="24" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="19" t="n">
+      <c r="B26" s="23" t="n">
         <v>50000</v>
       </c>
-      <c r="C26" s="20" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
+      <c r="C26" s="24" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B27" s="23" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C27" s="24" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="B29" s="19" t="n">
-        <v>624512</v>
-      </c>
-      <c r="C29" s="20" t="s">
-        <v>71</v>
-      </c>
+      <c r="A29" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B30" s="19" t="n">
-        <v>3099712</v>
-      </c>
-      <c r="C30" s="20" t="s">
-        <v>73</v>
+        <v>76</v>
+      </c>
+      <c r="B30" s="23" t="n">
+        <v>624512</v>
+      </c>
+      <c r="C30" s="24" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B31" s="19" t="n">
-        <v>605464</v>
-      </c>
-      <c r="C31" s="20" t="s">
-        <v>75</v>
+        <v>78</v>
+      </c>
+      <c r="B31" s="23" t="n">
+        <v>3099712</v>
+      </c>
+      <c r="C31" s="24" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B32" s="19" t="n">
-        <v>3053216</v>
-      </c>
-      <c r="C32" s="20" t="s">
-        <v>77</v>
+        <v>80</v>
+      </c>
+      <c r="B32" s="23" t="n">
+        <v>605464</v>
+      </c>
+      <c r="C32" s="24" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B33" s="18" t="n">
+        <v>82</v>
+      </c>
+      <c r="B33" s="23" t="n">
+        <v>3053216</v>
+      </c>
+      <c r="C33" s="24" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B34" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="C33" s="20" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
+      <c r="C34" s="24" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B36" s="19" t="n">
-        <v>690200</v>
-      </c>
-      <c r="C36" s="20" t="s">
-        <v>82</v>
-      </c>
+      <c r="A36" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B37" s="19" t="n">
+        <v>87</v>
+      </c>
+      <c r="B37" s="23" t="n">
+        <v>690200</v>
+      </c>
+      <c r="C37" s="24" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B38" s="23" t="n">
         <v>1428000</v>
       </c>
-      <c r="C37" s="20" t="s">
-        <v>84</v>
+      <c r="C38" s="24" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1597,8 +1698,8 @@
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A36:C36"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Corrige alerta de duplicacion (descartada con GPS, queda como falta de num_guia)
</commit_message>
<xml_diff>
--- a/finanzas/informes_semanales/Informe_Financiero_Semanal_Global_Solutions_07Ago2026.xlsx
+++ b/finanzas/informes_semanales/Informe_Financiero_Semanal_Global_Solutions_07Ago2026.xlsx
@@ -170,10 +170,10 @@
     <t xml:space="preserve">TOTAL SIN PAGAR</t>
   </si>
   <si>
-    <t xml:space="preserve">⚠ ALERTA — POSIBLE DUPLICACIÓN DE SERVICIOS (sin confirmar, revisar con OPE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Al cruzar contra GPS real (export de eventos trip/stop), se encontró que varios pares de servicios comparten el MISMO camión, MISMO día, MISMA ruta continua sin regreso a base entre uno y otro — ej. S-111/S-112 (Trans Luciano, Codegua, $210.000 c/u, ambos sin num_guia) y 8 servicios distintos con destino "Lampa" a exactamente $306.415 cada uno, también sin num_guia que los distinga. No se puede confirmar si son viajes reales separados o el mismo dato cargado más de una vez. El Total de Ventas de Agosto ($9.397.512) queda marcado como NO CONFIRMADO hasta que se revise.</t>
+    <t xml:space="preserve">⚠ NOTA — FALTA num_guia EN VARIOS SERVICIOS (no es duplicación, ya descartada con GPS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se revisó con GPS real (export de eventos trip/stop) el patrón de pares de servicios que compartían camión, día y monto (ej. S-111/S-112 Trans Luciano-Codegua; 8 servicios destino Lampa a $306.415). El GPS confirma que son viajes reales SEPARADOS — ida y vuelta corta, ventanas horarias distintas, sin pasar por base entre uno y otro, patrón normal para 2 servicios/día en tramos cortos. Descartada la duplicación. Pendiente real: estos servicios no tienen `num_guia` cargado en el sistema — falta trazabilidad documental, no es un error de conteo.</t>
   </si>
   <si>
     <t xml:space="preserve">NOTA IMPORTANTE</t>
@@ -388,10 +388,9 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <i val="true"/>
       <sz val="9"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FF9C6500"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -574,7 +573,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -617,10 +616,10 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF9C0006"/>
+      <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF9C6500"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>

</xml_diff>